<commit_message>
Add initial analysis notebook and results file for 4PT framework evaluation
- Created a new Jupyter notebook `norag_bak_1005.ipynb` containing the implementation of the 4PT analysis framework, including code for reading documents, processing data, and generating analysis results.
- Added a results file `analysis_results_20251005_225740.xlsx` to store the output of the analysis.
</commit_message>
<xml_diff>
--- a/data/processed/JRGsamples/JRG article sublist.xlsx
+++ b/data/processed/JRGsamples/JRG article sublist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinby/Library/CloudStorage/GoogleDrive-letheon.by@gmail.com/My Drive/AI44PT/Data/Processed Data/JRG samples/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xinby/Desktop/AI44PT_Desktop/data/processed/JRGsamples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BCDA43-2D41-5742-BFBD-00A150E62299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C52619E1-3D02-5643-BF84-DDC35D1D318C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{04FA40AC-F656-DF48-B52C-5210863698DE}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14400" windowHeight="18000" xr2:uid="{04FA40AC-F656-DF48-B52C-5210863698DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -156,21 +156,12 @@
     <t>Genia Kostka</t>
   </si>
   <si>
-    <t>Does the article fit in the universe of sustainability analyses we seek to assess? (Yes / No)</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>What problems or set of problems is the article trying to address?</t>
-  </si>
-  <si>
-    <t>Do the analysis, conclusions, and theories derived from, and directed to, understanding and/or managing a clearly specified "on the ground" problem or class of problems? (Yes / No)</t>
-  </si>
-  <si>
     <t>Interaction of program design conditions in affecting performance of voluntary programs</t>
   </si>
   <si>
@@ -202,21 +193,6 @@
   </si>
   <si>
     <t>Problems associated with China's environmental target system (target ridigity etc) that cause gap between regulatory goals and outcomes</t>
-  </si>
-  <si>
-    <t>Provide arguments that supports your response to Column U</t>
-  </si>
-  <si>
-    <t>Provide some key text passages from the article that support your response to Column U</t>
-  </si>
-  <si>
-    <t>Are the analysis, conclusions, and theories generated to apply beyond understanding, and/or managing a clearly specified “on the ground” problem or class of problems? (Yes / No)</t>
-  </si>
-  <si>
-    <t>Provide arguments that supports your response to Column X</t>
-  </si>
-  <si>
-    <t>Provide some key text passages from the article that support your response to Column X</t>
   </si>
   <si>
     <t>Geographical focus in several countries with no clearly specified on the ground problem</t>
@@ -351,24 +327,6 @@
     <t>Analysis result (based on column U and X)</t>
   </si>
   <si>
-    <t>Do the analysis, conclusions, and theories treat individuals, organizations and states as largely self-interested, satisfaction driven entities that seek to maximize some kind “utility” outcome? (Yes / No)</t>
-  </si>
-  <si>
-    <t>Provide arguments that supports your response to Column AB</t>
-  </si>
-  <si>
-    <t>Provide some key text passages from the article that support your response to Column AB</t>
-  </si>
-  <si>
-    <t>Do the analysis incorporate theories and conclusions incorporate an assessment of individuals, organizations and/or states that extends beyond self-interested satisfaction seeking motivations? (Yes / No)</t>
-  </si>
-  <si>
-    <t>Provide arguments that supports your response to Column AE</t>
-  </si>
-  <si>
-    <t>Provide some key text passages from the article that support your response to Column AE</t>
-  </si>
-  <si>
     <t>Analysis result (based on column AB and AE)</t>
   </si>
   <si>
@@ -496,15 +454,9 @@
     <t>Another highly salient aspect of the Chinese approach is the embedding of environmental targets in the cadre management system, which comprises a strong incentive system. At each administrative level, binding environmental targets are linked to government ofﬁcials’ annual evaluations that are the basis for promotion and bonus decisions. Without such a strict human resource management system, local implementers would be unlikely to heed environmental targets so closely. However, there are considerable downsides to the ubiquity of the Leninist state for environmental protection. The comparative literature from Global South countries shows that regulation can be improved by giving courts and prosecutors larger roles. In Brazil, prosecutors were very effective in initiating civil litigation against polluters (Shi &amp; Van Rooij 2014). While prosecutorial civil litigation has served environmental objectives in other countries in the Global South, in China, prosecutors are themselves subject to the very same target-based incentive system described in this paper, meaning that their capacity to push for change is limited. These differences highlight the importance of paying close attention to institutional settings when devising regulatory responses and looking to the opportunities offered by juridical tradition and local societal and political structures.</t>
   </si>
   <si>
-    <t>Final problem type of the article (Type 1, 2, 3, and 4)</t>
-  </si>
-  <si>
     <t>Problem type of the article (Type 1, 2, 3, and 4 autopopulated based on response to column U and AB)</t>
   </si>
   <si>
-    <t>Difficulty in coding the article and identifying the problem type (ambiguity of the article)</t>
-  </si>
-  <si>
     <t>Type 2</t>
   </si>
   <si>
@@ -533,6 +485,54 @@
   </si>
   <si>
     <t>Command without control: The case of China’s environmental target system</t>
+  </si>
+  <si>
+    <t>[Q1]Does the article fit in the universe of sustainability analyses we seek to assess? (Yes / No)</t>
+  </si>
+  <si>
+    <t>[Q2]What problems or set of problems is the article trying to address?</t>
+  </si>
+  <si>
+    <t>[Q3]Do the analysis, conclusions, and theories derived from, and directed to, understanding and/or managing a clearly specified "on the ground" problem or class of problems? (Yes / No)</t>
+  </si>
+  <si>
+    <t>[Q4]Provide arguments that supports your response to Column U</t>
+  </si>
+  <si>
+    <t>[Q5]Provide some key text passages from the article that support your response to Column U</t>
+  </si>
+  <si>
+    <t>[Q6]Are the analysis, conclusions, and theories generated to apply beyond understanding, and/or managing a clearly specified “on the ground” problem or class of problems? (Yes / No)</t>
+  </si>
+  <si>
+    <t>[Q7]Provide arguments that supports your response to Column X</t>
+  </si>
+  <si>
+    <t>[Q8]Provide some key text passages from the article that support your response to Column X</t>
+  </si>
+  <si>
+    <t>[Q9]Do the analysis, conclusions, and theories treat individuals, organizations and states as largely self-interested, satisfaction driven entities that seek to maximize some kind “utility” outcome? (Yes / No)</t>
+  </si>
+  <si>
+    <t>[Q10]Provide arguments that supports your response to Column AB</t>
+  </si>
+  <si>
+    <t>[Q11]Provide some key text passages from the article that support your response to Column AB</t>
+  </si>
+  <si>
+    <t>[Q12]Do the analysis incorporate theories and conclusions incorporate an assessment of individuals, organizations and/or states that extends beyond self-interested satisfaction seeking motivations? (Yes / No)</t>
+  </si>
+  <si>
+    <t>[Q13]Provide arguments that supports your response to Column AE</t>
+  </si>
+  <si>
+    <t>[Q14]Provide some key text passages from the article that support your response to Column AE</t>
+  </si>
+  <si>
+    <t>[Q15]Final problem type of the article (Type 1, 2, 3, and 4)</t>
+  </si>
+  <si>
+    <t>[Q16]Difficulty in coding the article and identifying the problem type (ambiguity of the article)</t>
   </si>
 </sst>
 </file>
@@ -901,61 +901,61 @@
         <v>24</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>145</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>146</v>
       </c>
       <c r="G1" t="s">
-        <v>40</v>
+        <v>147</v>
       </c>
       <c r="H1" t="s">
-        <v>52</v>
+        <v>148</v>
       </c>
       <c r="I1" t="s">
-        <v>53</v>
+        <v>149</v>
       </c>
       <c r="J1" t="s">
-        <v>54</v>
+        <v>150</v>
       </c>
       <c r="K1" t="s">
-        <v>55</v>
+        <v>151</v>
       </c>
       <c r="L1" t="s">
-        <v>56</v>
+        <v>152</v>
       </c>
       <c r="M1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="N1" t="s">
-        <v>100</v>
+        <v>153</v>
       </c>
       <c r="O1" t="s">
-        <v>101</v>
+        <v>154</v>
       </c>
       <c r="P1" t="s">
-        <v>102</v>
+        <v>155</v>
       </c>
       <c r="Q1" t="s">
-        <v>103</v>
+        <v>156</v>
       </c>
       <c r="R1" t="s">
-        <v>104</v>
+        <v>157</v>
       </c>
       <c r="S1" t="s">
-        <v>105</v>
+        <v>158</v>
       </c>
       <c r="T1" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="U1" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="V1" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="W1" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.2">
@@ -972,58 +972,58 @@
         <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="J2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="L2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="M2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O2" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="P2" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="Q2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R2" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="S2" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="T2" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U2" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="W2" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
@@ -1040,58 +1040,58 @@
         <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="I3" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="J3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K3" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="L3" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="M3" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O3" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="P3" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="Q3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R3" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="S3" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="T3" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U3" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="W3" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
@@ -1108,61 +1108,61 @@
         <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H4" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="I4" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="J4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K4" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="L4" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="M4" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O4" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="P4" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="Q4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R4" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="S4" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="T4" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U4" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="V4" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="W4" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.2">
@@ -1179,58 +1179,58 @@
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="G5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H5" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="I5" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="J5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K5" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="L5" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="M5" t="s">
+        <v>93</v>
+      </c>
+      <c r="N5" t="s">
+        <v>37</v>
+      </c>
+      <c r="O5" t="s">
+        <v>105</v>
+      </c>
+      <c r="P5" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>36</v>
+      </c>
+      <c r="R5" t="s">
         <v>107</v>
       </c>
-      <c r="N5" t="s">
-        <v>38</v>
-      </c>
-      <c r="O5" t="s">
-        <v>119</v>
-      </c>
-      <c r="P5" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>37</v>
-      </c>
-      <c r="R5" t="s">
-        <v>121</v>
-      </c>
       <c r="S5" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="T5" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U5" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="W5" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
@@ -1247,58 +1247,58 @@
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="I6" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="J6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K6" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="L6" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="M6" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O6" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="P6" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="Q6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R6" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="S6" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="T6" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U6" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="W6" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
@@ -1315,58 +1315,58 @@
         <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="I7" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="J7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="L7" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="M7" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O7" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="P7" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="Q7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="R7" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="S7" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="T7" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U7" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="W7" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
@@ -1383,58 +1383,58 @@
         <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H8" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I8" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="J8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K8" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="L8" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="M8" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O8" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="P8" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="Q8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R8" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="S8" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="T8" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U8" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="W8" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
@@ -1451,58 +1451,58 @@
         <v>32</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H9" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="I9" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="J9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K9" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="L9" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="M9" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O9" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="P9" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="Q9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R9" t="s">
+        <v>123</v>
+      </c>
+      <c r="S9" t="s">
+        <v>79</v>
+      </c>
+      <c r="T9" t="s">
+        <v>93</v>
+      </c>
+      <c r="U9" t="s">
         <v>137</v>
       </c>
-      <c r="S9" t="s">
-        <v>87</v>
-      </c>
-      <c r="T9" t="s">
-        <v>107</v>
-      </c>
-      <c r="U9" t="s">
-        <v>153</v>
-      </c>
       <c r="W9" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.2">
@@ -1519,58 +1519,58 @@
         <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H10" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="J10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K10" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="L10" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="M10" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O10" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="P10" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="Q10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R10" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="S10" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="T10" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U10" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="W10" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
@@ -1587,58 +1587,58 @@
         <v>34</v>
       </c>
       <c r="E11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H11" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="I11" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K11" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="L11" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="M11" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O11" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="P11" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="Q11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R11" t="s">
+        <v>128</v>
+      </c>
+      <c r="S11" t="s">
+        <v>129</v>
+      </c>
+      <c r="T11" t="s">
+        <v>93</v>
+      </c>
+      <c r="U11" t="s">
+        <v>137</v>
+      </c>
+      <c r="W11" t="s">
         <v>142</v>
-      </c>
-      <c r="S11" t="s">
-        <v>143</v>
-      </c>
-      <c r="T11" t="s">
-        <v>107</v>
-      </c>
-      <c r="U11" t="s">
-        <v>153</v>
-      </c>
-      <c r="W11" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
@@ -1649,67 +1649,67 @@
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="D12" t="s">
         <v>35</v>
       </c>
       <c r="E12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="G12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="I12" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="J12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K12" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="L12" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="M12" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="N12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O12" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="P12" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="Q12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R12" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="S12" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="T12" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="U12" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="V12" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="W12" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>